<commit_message>
update bug and validasi field
</commit_message>
<xml_diff>
--- a/uploads/excel/template_banksampah.xlsx
+++ b/uploads/excel/template_banksampah.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\igowi\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\kuliah\banksampahnew\uploads\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9CEAD7FD-9941-423C-BD3C-C48F8D1329F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31BE1EA5-B694-43EB-9DD7-27920847284C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{FA7A3973-2D5A-4D1F-BEB5-EC60649E320A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FA7A3973-2D5A-4D1F-BEB5-EC60649E320A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>No</t>
   </si>
@@ -58,6 +58,9 @@
   </si>
   <si>
     <t>alamat</t>
+  </si>
+  <si>
+    <t>nama_lengkap</t>
   </si>
 </sst>
 </file>
@@ -431,19 +434,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A919F892-BDD1-4F24-B589-42C8177EB39D}">
-  <dimension ref="A1:H31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I31"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.44140625" customWidth="1"/>
-    <col min="3" max="3" width="16.21875" customWidth="1"/>
-    <col min="4" max="4" width="17.6640625" customWidth="1"/>
-    <col min="5" max="5" width="15.88671875" customWidth="1"/>
-    <col min="6" max="6" width="18.21875" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" customWidth="1"/>
-    <col min="8" max="8" width="16.33203125" customWidth="1"/>
+    <col min="2" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.85546875" customWidth="1"/>
+    <col min="7" max="7" width="18.28515625" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" customWidth="1"/>
+    <col min="9" max="9" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -451,198 +454,201 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
         <f>A2+1</f>
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
-        <f t="shared" ref="A4:A34" si="0">A3+1</f>
+        <f t="shared" ref="A4:A31" si="0">A3+1</f>
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31">
         <f t="shared" si="0"/>
         <v>30</v>

</xml_diff>